<commit_message>
Improved backend + mobile responsiveness + new filters and reports
</commit_message>
<xml_diff>
--- a/sample_marks.xlsx
+++ b/sample_marks.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Marks Roster" sheetId="1" r:id="rId1"/>
+    <sheet name="Marks" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,220 +397,111 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Roll No</v>
+        <v>Student ID</v>
       </c>
       <c r="B1" t="str">
-        <v>Name</v>
+        <v>Student Name</v>
       </c>
       <c r="C1" t="str">
-        <v>Marks</v>
+        <v>IA1 (20)</v>
+      </c>
+      <c r="D1" t="str">
+        <v>IA2 (20)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Assignment 1</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Assignment 2</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>CS21B001</v>
+        <v>1HC24CS001</v>
       </c>
       <c r="B2" t="str">
         <v>Aakash Nair</v>
       </c>
       <c r="C2">
-        <v>42</v>
+        <v>18</v>
+      </c>
+      <c r="D2">
+        <v>19</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Yes</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>CS21B002</v>
+        <v>1HC24CS002</v>
       </c>
       <c r="B3" t="str">
         <v>Aditi Rao</v>
       </c>
       <c r="C3">
-        <v>45</v>
+        <v>15</v>
+      </c>
+      <c r="D3">
+        <v>16</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F3" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>CS21B003</v>
+        <v>1HC24CS003</v>
       </c>
       <c r="B4" t="str">
         <v>Ajay Singh</v>
       </c>
       <c r="C4">
-        <v>38</v>
+        <v>12</v>
+      </c>
+      <c r="D4">
+        <v>14</v>
+      </c>
+      <c r="E4" t="str">
+        <v>No</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Yes</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>CS21B004</v>
+        <v>1HC24CS004</v>
       </c>
       <c r="B5" t="str">
         <v>Amrita Das</v>
       </c>
       <c r="C5">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>CS21B005</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Ananya Krishnan</v>
-      </c>
-      <c r="C6">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>CS21B007</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Bhavna Pillai</v>
-      </c>
-      <c r="C7">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>CS21B008</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Deepak Verma</v>
-      </c>
-      <c r="C8">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>CS21B009</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Divya Sharma</v>
-      </c>
-      <c r="C9">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>CS21B010</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Ganesh Reddy</v>
-      </c>
-      <c r="C10">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>CS21B011</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Harish Kumar</v>
-      </c>
-      <c r="C11">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>CS21B012</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Ishita Bansal</v>
-      </c>
-      <c r="C12">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>CS21B013</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Jayant Patel</v>
-      </c>
-      <c r="C13">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>CS21B014</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Kavitha Mohan</v>
-      </c>
-      <c r="C14">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>CS21B015</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Kiran Menon</v>
-      </c>
-      <c r="C15">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>CS21B016</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Lavanya Subramanian</v>
-      </c>
-      <c r="C16">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>CS21B017</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Manish Gupta</v>
-      </c>
-      <c r="C17">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>CS21B018</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Rohit Sharma</v>
-      </c>
-      <c r="C18">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>CS21B042</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Rehman Dakait</v>
-      </c>
-      <c r="C19">
-        <v>48</v>
+        <v>20</v>
+      </c>
+      <c r="D5">
+        <v>18</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Yes</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>